<commit_message>
Edit header row in parameters; create sample_generate.py
</commit_message>
<xml_diff>
--- a/parameters.xlsx
+++ b/parameters.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mcgill-my.sharepoint.com/personal/meghana_munipalle_mail_mcgill_ca/Documents/research/ABM/RF sens materials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megmu\source\repos\megmuni\ABM-Random-Forest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="356" documentId="13_ncr:1_{2132A660-F15F-BD4F-9E31-F0FE3B728918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3ABB715D-FBE9-4A5F-8044-3FE1708D5807}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA0B3F8-D18E-4477-81C5-2A68B3250335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="792" yWindow="1596" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -46,12 +46,6 @@
     <t>SD</t>
   </si>
   <si>
-    <t>Lower limit</t>
-  </si>
-  <si>
-    <t>Upper limit</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
@@ -77,6 +71,12 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>Lower</t>
+  </si>
+  <si>
+    <t>Upper</t>
   </si>
 </sst>
 </file>
@@ -124,11 +124,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -463,16 +462,16 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
       <c r="G1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -496,10 +495,10 @@
         <v>4</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -526,7 +525,7 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -553,7 +552,7 @@
         <v>2</v>
       </c>
       <c r="J4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -580,7 +579,7 @@
         <v>3</v>
       </c>
       <c r="J5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -607,7 +606,7 @@
         <v>4</v>
       </c>
       <c r="J6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -684,10 +683,10 @@
         <f t="shared" si="0"/>
         <v>2.25</v>
       </c>
-      <c r="D10" s="3">
-        <v>1</v>
-      </c>
-      <c r="E10" s="3">
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
         <v>10</v>
       </c>
       <c r="F10">
@@ -820,7 +819,7 @@
         <v>1</v>
       </c>
       <c r="G16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -865,7 +864,7 @@
         <v>1</v>
       </c>
       <c r="G18" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -889,7 +888,7 @@
         <v>1</v>
       </c>
       <c r="G19" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -934,7 +933,7 @@
         <v>1</v>
       </c>
       <c r="G21" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -958,7 +957,7 @@
         <v>1</v>
       </c>
       <c r="G22" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
@@ -996,14 +995,14 @@
       <c r="D24" s="2">
         <v>10000</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="3">
         <v>1000000</v>
       </c>
       <c r="F24">
         <v>1</v>
       </c>
       <c r="G24" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1111,7 +1110,7 @@
         <v>4</v>
       </c>
       <c r="G29" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
@@ -1135,7 +1134,7 @@
         <v>4</v>
       </c>
       <c r="G30" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
@@ -1149,10 +1148,10 @@
         <f t="shared" si="0"/>
         <v>0.25</v>
       </c>
-      <c r="D31" s="3">
-        <v>0</v>
-      </c>
-      <c r="E31" s="3">
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
         <v>1</v>
       </c>
       <c r="F31">
@@ -1243,7 +1242,7 @@
         <v>1</v>
       </c>
       <c r="G35" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
@@ -1267,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="G36" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
@@ -1333,7 +1332,7 @@
         <v>1</v>
       </c>
       <c r="G39" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
@@ -1420,7 +1419,7 @@
         <v>1</v>
       </c>
       <c r="G43" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
@@ -1444,7 +1443,7 @@
         <v>1</v>
       </c>
       <c r="G44" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
@@ -1596,10 +1595,10 @@
         <v>1</v>
       </c>
       <c r="G51" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I51" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
@@ -1625,7 +1624,7 @@
         <v>1</v>
       </c>
       <c r="G52" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
@@ -1651,7 +1650,7 @@
         <v>1</v>
       </c>
       <c r="G53" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
@@ -1677,7 +1676,7 @@
         <v>1</v>
       </c>
       <c r="G54" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
@@ -1703,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="G55" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
@@ -1729,7 +1728,7 @@
         <v>1</v>
       </c>
       <c r="G56" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
@@ -1755,7 +1754,7 @@
         <v>1</v>
       </c>
       <c r="G57" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
@@ -1781,7 +1780,7 @@
         <v>1</v>
       </c>
       <c r="G58" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
@@ -1807,7 +1806,7 @@
         <v>1</v>
       </c>
       <c r="G59" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
@@ -1833,7 +1832,7 @@
         <v>1</v>
       </c>
       <c r="G60" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
@@ -1859,7 +1858,7 @@
         <v>1</v>
       </c>
       <c r="G61" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
@@ -1885,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="G62" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
@@ -1911,7 +1910,7 @@
         <v>1</v>
       </c>
       <c r="G63" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
@@ -1937,7 +1936,7 @@
         <v>1</v>
       </c>
       <c r="G64" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
@@ -1963,7 +1962,7 @@
         <v>1</v>
       </c>
       <c r="G65" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
@@ -1989,7 +1988,7 @@
         <v>1</v>
       </c>
       <c r="G66" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
@@ -2015,7 +2014,7 @@
         <v>1</v>
       </c>
       <c r="G67" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
@@ -2041,7 +2040,7 @@
         <v>1</v>
       </c>
       <c r="G68" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>